<commit_message>
Changes and correction - 22-10-2026
1. Correction in home page and accounts loan issue
2. Reports - show user mapped mappings.
3. Correction in loan track show loan issue user not account loan issue user.
4. Correction in Backoffice count report, mobile and direct unpaid not match with followed unpaid total.
5. correction in Bank statement upload excel format.
</commit_message>
<xml_diff>
--- a/uploads/excel_format/bank_stmt_format.xlsx
+++ b/uploads/excel_format/bank_stmt_format.xlsx
@@ -1,13 +1,8 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\marudham\uploads\excel_format\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="6" rupBuild="4505"/>
+  <workbookPr/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12435"/>
   </bookViews>
@@ -18,7 +13,7 @@
   <definedNames>
     <definedName name="AriyalurList">Sheet2!$E$2:$E$5</definedName>
     <definedName name="Bhuvanagiri">Sheet2!$H$2:$H$11</definedName>
-    <definedName name="BryanList">'Bank Statement'!$A$2:$A$7</definedName>
+    <definedName name="BryanList">'Bank Statement'!#REF!</definedName>
     <definedName name="ChennaiList">Sheet2!$F$2:$F$16</definedName>
     <definedName name="CoimbatoreList">Sheet2!$G$2:$G$12</definedName>
     <definedName name="CuddaloreList">Sheet2!$H$2:$H$11</definedName>
@@ -39,7 +34,7 @@
     <definedName name="PerambalurList">Sheet2!$T$2:$T$5</definedName>
     <definedName name="PondicherryList">Sheet2!$C$2:$C$5</definedName>
     <definedName name="PondicherryTalukList">Sheet2!#REF!</definedName>
-    <definedName name="ProductList">'Bank Statement'!$A$2:$A$7</definedName>
+    <definedName name="ProductList">'Bank Statement'!#REF!</definedName>
     <definedName name="PuducherryList">Sheet2!$AM$2:$AM$5</definedName>
     <definedName name="PudukkottaiList">Sheet2!$U$2:$U$13</definedName>
     <definedName name="RamanathapuramList">Sheet2!$V$2:$V$10</definedName>
@@ -62,9 +57,9 @@
     <definedName name="VirudhunagarList">Sheet2!$AJ$2:$AJ$11</definedName>
     <definedName name="YanamList">Sheet2!$AN$2:$AN$5</definedName>
   </definedNames>
-  <calcPr calcId="152511"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+  <calcPr calcId="124519"/>
+  <extLst xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -72,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="344">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="343">
   <si>
     <t>State</t>
   </si>
@@ -1089,9 +1084,6 @@
   </si>
   <si>
     <t>Date</t>
-  </si>
-  <si>
-    <t>Transaction ID</t>
   </si>
   <si>
     <t>Credit</t>
@@ -1109,8 +1101,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1153,15 +1145,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1225,7 +1212,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1260,7 +1247,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1437,659 +1424,39 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:XFD42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="16.85546875" customWidth="1"/>
-    <col min="3" max="3" width="38.28515625" customWidth="1"/>
-    <col min="4" max="4" width="20.140625" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" customWidth="1"/>
-    <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="15.28515625" customWidth="1"/>
-    <col min="9" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.140625" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" customWidth="1"/>
+    <col min="5" max="5" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16 16384:16384" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:5" s="2" customFormat="1">
+      <c r="A1" s="3" t="s">
         <v>338</v>
       </c>
-      <c r="B1" s="6" t="s">
-        <v>343</v>
-      </c>
-      <c r="C1" s="6" t="s">
+      <c r="B1" s="3" t="s">
+        <v>342</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>339</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="3" t="s">
         <v>340</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="3" t="s">
         <v>341</v>
       </c>
-      <c r="F1" s="6" t="s">
-        <v>342</v>
-      </c>
-      <c r="XFD1" s="5"/>
-    </row>
-    <row r="2" spans="1:16 16384:16384" x14ac:dyDescent="0.25">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2"/>
-      <c r="O2" s="2"/>
-      <c r="P2" s="2"/>
-    </row>
-    <row r="3" spans="1:16 16384:16384" x14ac:dyDescent="0.25">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
-      <c r="M3" s="2"/>
-      <c r="N3" s="2"/>
-      <c r="O3" s="2"/>
-      <c r="P3" s="2"/>
-    </row>
-    <row r="4" spans="1:16 16384:16384" x14ac:dyDescent="0.25">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-      <c r="M4" s="2"/>
-      <c r="N4" s="2"/>
-      <c r="O4" s="2"/>
-      <c r="P4" s="2"/>
-    </row>
-    <row r="5" spans="1:16 16384:16384" x14ac:dyDescent="0.25">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
-      <c r="L5" s="2"/>
-      <c r="M5" s="2"/>
-      <c r="N5" s="2"/>
-      <c r="O5" s="2"/>
-      <c r="P5" s="2"/>
-    </row>
-    <row r="6" spans="1:16 16384:16384" x14ac:dyDescent="0.25">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
-      <c r="K6" s="2"/>
-      <c r="L6" s="2"/>
-      <c r="M6" s="2"/>
-      <c r="N6" s="2"/>
-      <c r="O6" s="2"/>
-      <c r="P6" s="2"/>
-    </row>
-    <row r="7" spans="1:16 16384:16384" x14ac:dyDescent="0.25">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
-      <c r="L7" s="2"/>
-      <c r="M7" s="2"/>
-      <c r="N7" s="2"/>
-      <c r="O7" s="2"/>
-      <c r="P7" s="2"/>
-    </row>
-    <row r="8" spans="1:16 16384:16384" x14ac:dyDescent="0.25">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
-      <c r="N8" s="2"/>
-      <c r="O8" s="2"/>
-      <c r="P8" s="2"/>
-    </row>
-    <row r="9" spans="1:16 16384:16384" x14ac:dyDescent="0.25">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
-      <c r="L9" s="2"/>
-      <c r="M9" s="2"/>
-      <c r="N9" s="2"/>
-      <c r="O9" s="2"/>
-      <c r="P9" s="2"/>
-    </row>
-    <row r="10" spans="1:16 16384:16384" x14ac:dyDescent="0.25">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
-      <c r="J10" s="2"/>
-      <c r="K10" s="2"/>
-      <c r="L10" s="2"/>
-      <c r="M10" s="2"/>
-      <c r="N10" s="2"/>
-      <c r="O10" s="2"/>
-      <c r="P10" s="2"/>
-    </row>
-    <row r="11" spans="1:16 16384:16384" x14ac:dyDescent="0.25">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2"/>
-      <c r="K11" s="2"/>
-      <c r="L11" s="2"/>
-      <c r="M11" s="2"/>
-      <c r="N11" s="2"/>
-      <c r="O11" s="2"/>
-      <c r="P11" s="2"/>
-    </row>
-    <row r="12" spans="1:16 16384:16384" x14ac:dyDescent="0.25">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
-      <c r="J12" s="2"/>
-      <c r="K12" s="2"/>
-      <c r="L12" s="2"/>
-      <c r="M12" s="2"/>
-      <c r="N12" s="2"/>
-      <c r="O12" s="2"/>
-      <c r="P12" s="2"/>
-    </row>
-    <row r="13" spans="1:16 16384:16384" x14ac:dyDescent="0.25">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
-      <c r="L13" s="2"/>
-      <c r="M13" s="2"/>
-      <c r="N13" s="2"/>
-      <c r="O13" s="2"/>
-      <c r="P13" s="2"/>
-    </row>
-    <row r="14" spans="1:16 16384:16384" x14ac:dyDescent="0.25">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
-      <c r="J14" s="2"/>
-      <c r="K14" s="2"/>
-      <c r="L14" s="2"/>
-      <c r="M14" s="2"/>
-      <c r="N14" s="2"/>
-      <c r="O14" s="2"/>
-      <c r="P14" s="2"/>
-    </row>
-    <row r="15" spans="1:16 16384:16384" x14ac:dyDescent="0.25">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
-      <c r="J15" s="2"/>
-      <c r="K15" s="2"/>
-      <c r="L15" s="2"/>
-      <c r="M15" s="2"/>
-      <c r="N15" s="2"/>
-      <c r="O15" s="2"/>
-      <c r="P15" s="2"/>
-    </row>
-    <row r="16" spans="1:16 16384:16384" x14ac:dyDescent="0.25">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
-      <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
-      <c r="L16" s="2"/>
-      <c r="M16" s="2"/>
-      <c r="N16" s="2"/>
-      <c r="O16" s="2"/>
-      <c r="P16" s="2"/>
-    </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
-      <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
-      <c r="J17" s="2"/>
-      <c r="K17" s="2"/>
-      <c r="L17" s="2"/>
-      <c r="M17" s="2"/>
-      <c r="N17" s="2"/>
-      <c r="O17" s="2"/>
-      <c r="P17" s="2"/>
-    </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
-      <c r="H18" s="2"/>
-      <c r="I18" s="2"/>
-      <c r="J18" s="2"/>
-      <c r="K18" s="2"/>
-      <c r="L18" s="2"/>
-      <c r="M18" s="2"/>
-      <c r="N18" s="2"/>
-      <c r="O18" s="2"/>
-      <c r="P18" s="2"/>
-    </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="2"/>
-      <c r="I19" s="2"/>
-      <c r="J19" s="2"/>
-      <c r="K19" s="2"/>
-      <c r="L19" s="2"/>
-      <c r="M19" s="2"/>
-      <c r="N19" s="2"/>
-      <c r="O19" s="2"/>
-      <c r="P19" s="2"/>
-    </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
-      <c r="H20" s="2"/>
-      <c r="I20" s="2"/>
-      <c r="J20" s="2"/>
-      <c r="K20" s="2"/>
-      <c r="L20" s="2"/>
-      <c r="M20" s="2"/>
-      <c r="N20" s="2"/>
-      <c r="O20" s="2"/>
-      <c r="P20" s="2"/>
-    </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
-      <c r="H21" s="2"/>
-      <c r="I21" s="2"/>
-      <c r="J21" s="2"/>
-      <c r="K21" s="2"/>
-      <c r="L21" s="2"/>
-      <c r="M21" s="2"/>
-      <c r="N21" s="2"/>
-      <c r="O21" s="2"/>
-      <c r="P21" s="2"/>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A22" s="2"/>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
-      <c r="H22" s="2"/>
-      <c r="I22" s="2"/>
-      <c r="J22" s="2"/>
-      <c r="K22" s="2"/>
-      <c r="L22" s="2"/>
-      <c r="M22" s="2"/>
-      <c r="N22" s="2"/>
-      <c r="O22" s="2"/>
-      <c r="P22" s="2"/>
-    </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A23" s="2"/>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="2"/>
-      <c r="I23" s="2"/>
-      <c r="J23" s="2"/>
-      <c r="K23" s="2"/>
-      <c r="L23" s="2"/>
-      <c r="M23" s="2"/>
-      <c r="N23" s="2"/>
-      <c r="O23" s="2"/>
-      <c r="P23" s="2"/>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A24" s="2"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
-      <c r="H24" s="2"/>
-      <c r="I24" s="2"/>
-      <c r="J24" s="2"/>
-      <c r="K24" s="2"/>
-      <c r="L24" s="2"/>
-      <c r="M24" s="2"/>
-      <c r="N24" s="2"/>
-      <c r="O24" s="2"/>
-      <c r="P24" s="2"/>
-    </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A25" s="2"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
-      <c r="H25" s="2"/>
-      <c r="I25" s="2"/>
-      <c r="J25" s="2"/>
-      <c r="K25" s="2"/>
-      <c r="L25" s="2"/>
-      <c r="M25" s="2"/>
-      <c r="N25" s="2"/>
-      <c r="O25" s="2"/>
-      <c r="P25" s="2"/>
-    </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A26" s="2"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
-      <c r="H26" s="2"/>
-      <c r="I26" s="2"/>
-    </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A27" s="2"/>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
-      <c r="H27" s="2"/>
-      <c r="I27" s="2"/>
-    </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A28" s="2"/>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
-      <c r="H28" s="2"/>
-      <c r="I28" s="2"/>
-    </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A29" s="2"/>
-      <c r="B29" s="2"/>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
-      <c r="F29" s="2"/>
-      <c r="G29" s="2"/>
-      <c r="H29" s="2"/>
-      <c r="I29" s="2"/>
-    </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A30" s="2"/>
-      <c r="B30" s="2"/>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="2"/>
-      <c r="G30" s="2"/>
-      <c r="H30" s="2"/>
-      <c r="I30" s="2"/>
-    </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A31" s="2"/>
-      <c r="B31" s="2"/>
-      <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
-      <c r="E31" s="2"/>
-      <c r="F31" s="2"/>
-      <c r="G31" s="2"/>
-      <c r="H31" s="2"/>
-      <c r="I31" s="2"/>
-    </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A32" s="2"/>
-      <c r="B32" s="2"/>
-      <c r="C32" s="2"/>
-      <c r="D32" s="2"/>
-      <c r="E32" s="2"/>
-      <c r="F32" s="2"/>
-      <c r="G32" s="2"/>
-      <c r="H32" s="2"/>
-      <c r="I32" s="2"/>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="2"/>
-      <c r="B33" s="2"/>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
-      <c r="F33" s="2"/>
-      <c r="G33" s="2"/>
-      <c r="H33" s="2"/>
-      <c r="I33" s="2"/>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A34" s="2"/>
-      <c r="B34" s="2"/>
-      <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
-      <c r="E34" s="2"/>
-      <c r="F34" s="2"/>
-      <c r="G34" s="2"/>
-      <c r="H34" s="2"/>
-      <c r="I34" s="2"/>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A35" s="2"/>
-      <c r="B35" s="2"/>
-      <c r="C35" s="2"/>
-      <c r="D35" s="2"/>
-      <c r="E35" s="2"/>
-      <c r="F35" s="2"/>
-      <c r="G35" s="2"/>
-      <c r="H35" s="2"/>
-      <c r="I35" s="2"/>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A36" s="2"/>
-      <c r="B36" s="2"/>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
-      <c r="E36" s="2"/>
-      <c r="F36" s="2"/>
-      <c r="G36" s="2"/>
-      <c r="H36" s="2"/>
-      <c r="I36" s="2"/>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A37" s="2"/>
-      <c r="B37" s="2"/>
-      <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
-      <c r="E37" s="2"/>
-      <c r="F37" s="2"/>
-      <c r="G37" s="2"/>
-      <c r="H37" s="2"/>
-      <c r="I37" s="2"/>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A38" s="2"/>
-      <c r="B38" s="2"/>
-      <c r="C38" s="2"/>
-      <c r="D38" s="2"/>
-      <c r="E38" s="2"/>
-      <c r="F38" s="2"/>
-      <c r="G38" s="2"/>
-      <c r="H38" s="2"/>
-      <c r="I38" s="2"/>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A39" s="2"/>
-      <c r="B39" s="2"/>
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
-      <c r="E39" s="2"/>
-      <c r="F39" s="2"/>
-      <c r="G39" s="2"/>
-      <c r="H39" s="2"/>
-      <c r="I39" s="2"/>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A40" s="3"/>
-      <c r="B40" s="3"/>
-      <c r="C40" s="3"/>
-      <c r="D40" s="3"/>
-      <c r="E40" s="3"/>
-      <c r="F40" s="3"/>
-      <c r="G40" s="3"/>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A41" s="3"/>
-      <c r="B41" s="3"/>
-      <c r="C41" s="3"/>
-      <c r="D41" s="3"/>
-      <c r="E41" s="3"/>
-      <c r="F41" s="3"/>
-      <c r="G41" s="3"/>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A42" s="3"/>
-      <c r="B42" s="3"/>
-      <c r="C42" s="3"/>
-      <c r="D42" s="3"/>
-      <c r="E42" s="3"/>
-      <c r="F42" s="3"/>
-      <c r="G42" s="3"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
@@ -2099,15 +1466,15 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AO33"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:41">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2226,7 +1593,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="2" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:41">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -2345,7 +1712,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="3" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:41">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -2464,7 +1831,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="4" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:41">
       <c r="B4" t="s">
         <v>6</v>
       </c>
@@ -2580,7 +1947,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:41">
       <c r="B5" t="s">
         <v>7</v>
       </c>
@@ -2696,7 +2063,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="6" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:41">
       <c r="B6" t="s">
         <v>8</v>
       </c>
@@ -2791,7 +2158,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="7" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:41">
       <c r="B7" t="s">
         <v>9</v>
       </c>
@@ -2880,7 +2247,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="8" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:41">
       <c r="B8" t="s">
         <v>10</v>
       </c>
@@ -2957,7 +2324,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="9" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:41">
       <c r="B9" t="s">
         <v>11</v>
       </c>
@@ -3031,7 +2398,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="10" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:41">
       <c r="B10" t="s">
         <v>12</v>
       </c>
@@ -3090,7 +2457,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="11" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:41">
       <c r="B11" t="s">
         <v>13</v>
       </c>
@@ -3131,7 +2498,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="12" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:41">
       <c r="B12" t="s">
         <v>14</v>
       </c>
@@ -3151,7 +2518,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="13" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:41">
       <c r="B13" t="s">
         <v>15</v>
       </c>
@@ -3168,7 +2535,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="14" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:41">
       <c r="B14" t="s">
         <v>16</v>
       </c>
@@ -3179,7 +2546,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="15" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:41">
       <c r="B15" t="s">
         <v>17</v>
       </c>
@@ -3187,7 +2554,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="16" spans="1:41" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:41">
       <c r="B16" t="s">
         <v>18</v>
       </c>
@@ -3195,93 +2562,93 @@
         <v>90</v>
       </c>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:2">
       <c r="B17" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:2">
       <c r="B18" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:2">
       <c r="B19" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:2">
       <c r="B20" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:2">
       <c r="B21" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:2">
       <c r="B22" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="23" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:2">
       <c r="B23" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:2">
       <c r="B24" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="25" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:2">
       <c r="B25" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="26" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:2">
       <c r="B26" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="27" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:2">
       <c r="B27" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="28" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:2">
       <c r="B28" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="29" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:2">
       <c r="B29" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="30" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:2">
       <c r="B30" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="31" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:2">
       <c r="B31" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="32" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:2">
       <c r="B32" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:2">
       <c r="B33" t="s">
         <v>35</v>
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="ipAETGhLPGHFyUJSaDN6RKsCH6Vb32QYdZIcgfJ/Am75J8Nvek/XWcIofmV9oo3FSuNmMyPZBTZ8YC/A4sY1rg==" saltValue="ujbtXg+61P/0HGyqWm1cFw==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>